<commit_message>
Update Imagine and test features
</commit_message>
<xml_diff>
--- a/EXTRA/test_features_ver1.xlsx
+++ b/EXTRA/test_features_ver1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WIN-LOR\Documents\LTM_CARO\Project\EXTRA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E6EAA43-C02C-41F2-BD4D-0F27F2579AD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D1268D4-5638-4599-823A-D59DD5B6AA75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,100 +35,8 @@
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
-  <metadataTypes count="1">
-    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="8">
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="0"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="1"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="2"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="3"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="4"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="5"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="6"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="7"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <valueMetadata count="8">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-    <bk>
-      <rc t="1" v="1"/>
-    </bk>
-    <bk>
-      <rc t="1" v="2"/>
-    </bk>
-    <bk>
-      <rc t="1" v="3"/>
-    </bk>
-    <bk>
-      <rc t="1" v="4"/>
-    </bk>
-    <bk>
-      <rc t="1" v="5"/>
-    </bk>
-    <bk>
-      <rc t="1" v="6"/>
-    </bk>
-    <bk>
-      <rc t="1" v="7"/>
-    </bk>
-  </valueMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t>No</t>
   </si>
@@ -251,6 +159,30 @@
   </si>
   <si>
     <t>Hiện bảng xếp theo tứ thứ tự điểm số</t>
+  </si>
+  <si>
+    <t>Imagine/Client_Server</t>
+  </si>
+  <si>
+    <t>Imagine/Challenge</t>
+  </si>
+  <si>
+    <t>Imagine/His</t>
+  </si>
+  <si>
+    <t>Imagine/Time</t>
+  </si>
+  <si>
+    <t>Imagine/chat</t>
+  </si>
+  <si>
+    <t>Imagine/WatchHis</t>
+  </si>
+  <si>
+    <t>Imagine/PlayAI</t>
+  </si>
+  <si>
+    <t>Imagine/BangXepHang</t>
   </si>
 </sst>
 </file>
@@ -351,7 +283,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -378,7 +310,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -394,105 +325,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
-<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
-  <global>
-    <keyFlags>
-      <key name="_Self">
-        <flag name="ExcludeFromFile" value="1"/>
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_DisplayString">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Flags">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Format">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_SubLabel">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Attribution">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Icon">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Display">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_CanonicalPropertyNames">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_ClassificationId">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-    </keyFlags>
-  </global>
-</rvTypesInfo>
-</file>
-
-<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="8">
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>1</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>2</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>3</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>4</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>5</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>6</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>7</v>
-    <v>5</v>
-  </rv>
-</rvData>
-</file>
-
-<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <s t="_localImage">
-    <k n="_rvRel:LocalImageIdentifier" t="i"/>
-    <k n="CalcOrigin" t="i"/>
-  </s>
-</rvStructures>
-</file>
-
-<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
-<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <rel r:id="rId1"/>
-  <rel r:id="rId2"/>
-  <rel r:id="rId3"/>
-  <rel r:id="rId4"/>
-  <rel r:id="rId5"/>
-  <rel r:id="rId6"/>
-  <rel r:id="rId7"/>
-  <rel r:id="rId8"/>
-</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -828,8 +660,8 @@
       <c r="E2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="5" t="e" vm="1">
-        <v>#VALUE!</v>
+      <c r="F2" s="5" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="139.94999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -848,8 +680,8 @@
       <c r="E3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="5" t="e" vm="2">
-        <v>#VALUE!</v>
+      <c r="F3" s="5" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="139.94999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -868,8 +700,8 @@
       <c r="E4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="5" t="e" vm="3">
-        <v>#VALUE!</v>
+      <c r="F4" s="5" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="139.94999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -888,8 +720,8 @@
       <c r="E5" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="5" t="e" vm="4">
-        <v>#VALUE!</v>
+      <c r="F5" s="5" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="139.94999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -908,8 +740,8 @@
       <c r="E6" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="5" t="e" vm="5">
-        <v>#VALUE!</v>
+      <c r="F6" s="5" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="139.94999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -928,8 +760,8 @@
       <c r="E7" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="5" t="e" vm="6">
-        <v>#VALUE!</v>
+      <c r="F7" s="5" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="139.94999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -948,13 +780,13 @@
       <c r="E8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F8" s="5" t="e" vm="7">
-        <v>#VALUE!</v>
+      <c r="F8" s="5" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="139.94999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="8">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" s="8" t="s">
         <v>34</v>
@@ -968,8 +800,8 @@
       <c r="E9" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="10" t="e" vm="8">
-        <v>#VALUE!</v>
+      <c r="F9" s="5" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>